<commit_message>
n8n board refresh 2026-06-07T17:47:14Z
</commit_message>
<xml_diff>
--- a/app/reports/LDOS_research.xlsx
+++ b/app/reports/LDOS_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-06 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-07 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1694,10 +1694,10 @@
         <v>26.305511</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>16.786</v>
+        <v>16.919</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>4.593</v>
+        <v>4.603</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-26T17:39:13Z
</commit_message>
<xml_diff>
--- a/app/reports/LDOS_research.xlsx
+++ b/app/reports/LDOS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-18 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-26 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.697</v>
+        <v>0.702</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>107.055</v>
+        <v>101.135</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.868</v>
+        <v>0.885</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04438000202178955</v>
+        <v>0.04372000217437744</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>125785460.7071132</v>
+        <v>125785462.6785979</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>107.055</v>
+        <v>101.135</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>13465962496</v>
+        <v>12721312768</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.789999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.66</v>
+        <v>7.95</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>15838826496</v>
+        <v>16153994240</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>14.646524</v>
+        <v>14.937967</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>11.205</v>
+        <v>10.705</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>2.696</v>
+        <v>2.576</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>16394600448</v>
+        <v>16651383808</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.630938</v>
+        <v>15.875761</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>11.193</v>
+        <v>11.06</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.969</v>
+        <v>0.957</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>53144944640</v>
+        <v>55344971776</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>61.989315</v>
+        <v>65.10991</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>27.14</v>
+        <v>29.692</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.003</v>
+        <v>2.191</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>12769387520</v>
+        <v>13296078848</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>11.106558</v>
+        <v>11.779222</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>6.056</v>
+        <v>5.727</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>1.083</v>
+        <v>1.024</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>21367822336</v>
+        <v>20659066880</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>8.653703999999999</v>
+        <v>8.366667</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>6.234</v>
+        <v>5.968</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>0.512</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>8502220288</v>
+        <v>8911798272</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>12.560831</v>
+        <v>13.152915</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8.385999999999999</v>
+        <v>7.604</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>1.732</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="12">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>31276656640</v>
+        <v>29483988992</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>25.140158</v>
+        <v>23.699213</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>16.318</v>
+        <v>15.624</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>4.439</v>
+        <v>4.251</v>
       </c>
     </row>
     <row r="13">
@@ -1700,16 +1700,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>28620982272</v>
+        <v>29123885056</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>31.327335</v>
+        <v>31.81326</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>20.247</v>
+        <v>20.16</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>5.003</v>
+        <v>4.981</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-29T17:41:52Z
</commit_message>
<xml_diff>
--- a/app/reports/LDOS_research.xlsx
+++ b/app/reports/LDOS_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-21 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-29 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.736</v>
+        <v>0.726</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>104.71</v>
+        <v>115.67</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.875</v>
+        <v>0.844</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04625999927520752</v>
+        <v>0.04647000312805176</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>125785466.7558018</v>
+        <v>125785461.675456</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>104.71</v>
+        <v>115.67</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>13170996224</v>
+        <v>14549604352</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>9.58</v>
+        <v>10.59</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.32</v>
+        <v>8.91</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>1.15</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>16791270400</v>
+        <v>18590337024</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>15.527271</v>
+        <v>17.190908</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>11.608</v>
+        <v>12.144</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>2.793</v>
+        <v>2.922</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>16429731840</v>
+        <v>18827024384</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>15.6644335</v>
+        <v>17.95006</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>11.188</v>
+        <v>12.092</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>0.968</v>
+        <v>1.046</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>46824587264</v>
+        <v>37937807360</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>54.84979</v>
+        <v>44.439915</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>22.334</v>
+        <v>21.155</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>1.648</v>
+        <v>1.561</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>14022766592</v>
+        <v>15551533056</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>12.4</v>
+        <v>13.650736</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>6.157</v>
+        <v>6.383</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>1.101</v>
+        <v>1.142</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>22446958592</v>
+        <v>26100477952</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>9.09074</v>
+        <v>10.570371</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>6.22</v>
+        <v>7.01</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>0.51</v>
+        <v>0.575</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>8994122752</v>
+        <v>11084554240</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>13.287547</v>
+        <v>16.375866</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8.327</v>
+        <v>9.067</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>1.72</v>
+        <v>1.872</v>
       </c>
     </row>
     <row r="12">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>32205318144</v>
+        <v>34181167104</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>25.886616</v>
+        <v>27.474804</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>16.308</v>
+        <v>17.698</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>4.437</v>
+        <v>4.815</v>
       </c>
     </row>
     <row r="13">
@@ -1700,16 +1700,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>30579546112</v>
+        <v>29436606464</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>33.437183</v>
+        <v>30.754114</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>20.142</v>
+        <v>19.972</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.977</v>
+        <v>4.989</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-23T17:40:42Z
</commit_message>
<xml_diff>
--- a/app/reports/LDOS_research.xlsx
+++ b/app/reports/LDOS_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-23 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
         <v>40800559104</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>42.48077</v>
+        <v>42.810078</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>20.674</v>

</xml_diff>